<commit_message>
Some updates to the diagnostics program and the order sheet.
</commit_message>
<xml_diff>
--- a/Charge_Indicator/BOM and Order Sheet/Order_Sheet_REV2.xlsx
+++ b/Charge_Indicator/BOM and Order Sheet/Order_Sheet_REV2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathanfikes/Documents/GitHub/AutoNav-Charge_Indicator-KiCad_Pcb/Charge_Indicator/BOM and Order Sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4D1566-F3D8-B148-986C-90A86B1A9C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D52320-5DEF-0A47-B2C2-C2FED7C583CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17800" xr2:uid="{F977D430-13CE-AD47-96E5-85BBB755CDD5}"/>
+    <workbookView xWindow="9540" yWindow="660" windowWidth="20700" windowHeight="17800" xr2:uid="{F977D430-13CE-AD47-96E5-85BBB755CDD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="205">
   <si>
     <t>Qty</t>
   </si>
@@ -604,6 +604,123 @@
   </si>
   <si>
     <t>Actual Costs Breakdown: (REV2)</t>
+  </si>
+  <si>
+    <t>Ea.</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>0.005ΩSurge Resistor</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>0.01ΩSurge Resistor</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>10kΩThermistor</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>‎</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="游ゴシック"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>WSL25125L000FEA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>‎</t>
+    </r>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <r>
+      <t>WSL1206R0100JEA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>‎</t>
+    </r>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>‎</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="游ゴシック"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NCP18XH103D03RB</t>
+    </r>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>Digikey</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>Vishay Dale</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>Murata Electronics</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>490-11813-1-ND</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>541-WSL1206R0100JEACT-ND</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>WSLG-.005CT-ND</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/vishay-dale/WSL25125L000FEA/712555</t>
+    <phoneticPr fontId="6"/>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/vishay-dale/WSL1206R0100JEA/9752083</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/NCP18XH103D03RB/5773685?s=N4IgTCBcDaKHAEA5AwgBQIwA4AaAJNAGAZgBEiAlAIRAF0BfIA</t>
+    <phoneticPr fontId="6"/>
   </si>
 </sst>
 </file>
@@ -614,18 +731,18 @@
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="游ゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="游ゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -633,7 +750,7 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
-      <name val="Aptos Narrow"/>
+      <name val="游ゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -641,7 +758,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="游ゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -649,17 +766,45 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="游ゴシック"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="游ゴシック"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="游ゴシック"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -693,6 +838,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -859,7 +1010,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -957,6 +1108,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -966,6 +1118,36 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -975,42 +1157,18 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="ハイパーリンク" xfId="2" builtinId="8"/>
+    <cellStyle name="通貨 [0.00]" xfId="1" builtinId="4"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1031,7 +1189,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1347,21 +1505,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5429AA39-1145-AF43-8726-DB045179E867}">
-  <dimension ref="A2:P59"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A2:P62"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="23" customWidth="1"/>
-    <col min="13" max="13" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="133" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16">
       <c r="P2" s="19" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="76">
       <c r="A3" s="16" t="s">
         <v>52</v>
       </c>
@@ -1371,14 +1529,14 @@
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="48" t="s">
+      <c r="D3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="52"/>
       <c r="J3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1401,7 +1559,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="21">
       <c r="A4" s="26">
         <v>5</v>
       </c>
@@ -1412,14 +1570,14 @@
       <c r="C4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="49" t="s">
+      <c r="D4" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="51"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="50"/>
       <c r="J4" s="8" t="s">
         <v>14</v>
       </c>
@@ -1444,7 +1602,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="21">
       <c r="A5" s="27"/>
       <c r="B5" s="11">
         <f t="shared" ref="B5:B9" si="1">1*$A$4</f>
@@ -1453,14 +1611,14 @@
       <c r="C5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="49" t="s">
+      <c r="D5" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="51"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="50"/>
       <c r="J5" s="8" t="s">
         <v>20</v>
       </c>
@@ -1484,7 +1642,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="21">
       <c r="A6" s="27"/>
       <c r="B6" s="11">
         <f t="shared" si="1"/>
@@ -1493,14 +1651,14 @@
       <c r="C6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="49" t="s">
+      <c r="D6" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="51"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="50"/>
       <c r="J6" s="8" t="s">
         <v>26</v>
       </c>
@@ -1524,7 +1682,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="21">
       <c r="A7" s="27"/>
       <c r="B7" s="11">
         <f t="shared" si="1"/>
@@ -1533,14 +1691,14 @@
       <c r="C7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="49" t="s">
+      <c r="D7" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="51"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="50"/>
       <c r="J7" s="8" t="s">
         <v>27</v>
       </c>
@@ -1564,7 +1722,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="21">
       <c r="A8" s="27"/>
       <c r="B8" s="11">
         <f t="shared" si="1"/>
@@ -1573,14 +1731,14 @@
       <c r="C8" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="49" t="s">
+      <c r="D8" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="50"/>
-      <c r="F8" s="50"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="50"/>
-      <c r="I8" s="51"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="50"/>
       <c r="J8" s="8" t="s">
         <v>38</v>
       </c>
@@ -1604,7 +1762,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="21">
       <c r="A9" s="27"/>
       <c r="B9" s="11">
         <f t="shared" si="1"/>
@@ -1613,14 +1771,14 @@
       <c r="C9" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="49" t="s">
+      <c r="D9" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="50"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="51"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="50"/>
       <c r="J9" s="8" t="s">
         <v>44</v>
       </c>
@@ -1644,7 +1802,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" ht="21">
       <c r="A10" s="27"/>
       <c r="B10" s="11">
         <f>5*$A$4</f>
@@ -1653,14 +1811,14 @@
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="49" t="s">
+      <c r="D10" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="50"/>
-      <c r="F10" s="50"/>
-      <c r="G10" s="50"/>
-      <c r="H10" s="50"/>
-      <c r="I10" s="51"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="50"/>
       <c r="J10" s="8" t="s">
         <v>49</v>
       </c>
@@ -1684,7 +1842,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" ht="21">
       <c r="A11" s="27"/>
       <c r="B11" s="11">
         <f>8*$A$4</f>
@@ -1693,14 +1851,14 @@
       <c r="C11" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="49" t="s">
+      <c r="D11" s="48" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="51"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="49"/>
+      <c r="I11" s="50"/>
       <c r="J11" s="8" t="s">
         <v>55</v>
       </c>
@@ -1724,7 +1882,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" ht="21">
       <c r="A12" s="27"/>
       <c r="B12" s="11">
         <f>3*$A$4</f>
@@ -1733,14 +1891,14 @@
       <c r="C12" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="43"/>
+      <c r="I12" s="44"/>
       <c r="J12" s="8" t="s">
         <v>59</v>
       </c>
@@ -1764,7 +1922,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16">
       <c r="A13" s="27"/>
       <c r="B13" s="11">
         <f>1*$A$4</f>
@@ -1773,14 +1931,14 @@
       <c r="C13" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="43"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="43"/>
+      <c r="I13" s="44"/>
       <c r="J13" s="10" t="s">
         <v>61</v>
       </c>
@@ -1804,7 +1962,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" ht="21">
       <c r="A14" s="27"/>
       <c r="B14" s="11">
         <f>1*$A$4</f>
@@ -1813,14 +1971,14 @@
       <c r="C14" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="43"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="44"/>
       <c r="J14" s="8" t="s">
         <v>64</v>
       </c>
@@ -1844,7 +2002,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16">
       <c r="A15" s="27"/>
       <c r="B15" s="11">
         <f>1*$A$4</f>
@@ -1853,14 +2011,14 @@
       <c r="C15" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="41" t="s">
+      <c r="D15" s="42" t="s">
         <v>72</v>
       </c>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="43"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
+      <c r="H15" s="43"/>
+      <c r="I15" s="44"/>
       <c r="J15" s="10" t="s">
         <v>68</v>
       </c>
@@ -1884,7 +2042,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16">
       <c r="A16" s="27"/>
       <c r="B16" s="11">
         <v>0</v>
@@ -1892,14 +2050,14 @@
       <c r="C16" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="43"/>
+      <c r="I16" s="44"/>
       <c r="J16" s="10" t="s">
         <v>73</v>
       </c>
@@ -1923,7 +2081,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" ht="21">
       <c r="A17" s="27"/>
       <c r="B17" s="11">
         <f>1*$A$4</f>
@@ -1932,14 +2090,14 @@
       <c r="C17" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="49" t="s">
+      <c r="D17" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="E17" s="50"/>
-      <c r="F17" s="50"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="50"/>
-      <c r="I17" s="51"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="50"/>
       <c r="J17" s="8" t="s">
         <v>77</v>
       </c>
@@ -1963,7 +2121,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="21">
       <c r="A18" s="27"/>
       <c r="B18" s="11">
         <f>2*$A$4</f>
@@ -1972,14 +2130,14 @@
       <c r="C18" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="49" t="s">
+      <c r="D18" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="51"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="49"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="50"/>
       <c r="J18" s="8" t="s">
         <v>80</v>
       </c>
@@ -2003,7 +2161,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" ht="21">
       <c r="A19" s="27"/>
       <c r="B19" s="11">
         <f>2*$A$4</f>
@@ -2012,14 +2170,14 @@
       <c r="C19" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="42" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="42"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="43"/>
+      <c r="I19" s="44"/>
       <c r="J19" s="10" t="s">
         <v>86</v>
       </c>
@@ -2043,7 +2201,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16">
       <c r="A20" s="27"/>
       <c r="B20" s="11">
         <f>1*$A$4</f>
@@ -2052,14 +2210,14 @@
       <c r="C20" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="42" t="s">
         <v>92</v>
       </c>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="43"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="43"/>
+      <c r="I20" s="44"/>
       <c r="J20" s="10" t="s">
         <v>90</v>
       </c>
@@ -2083,7 +2241,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="21">
       <c r="A21" s="27"/>
       <c r="B21" s="11">
         <f>2*$A$4</f>
@@ -2092,14 +2250,14 @@
       <c r="C21" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="43"/>
+      <c r="I21" s="44"/>
       <c r="J21" s="8" t="s">
         <v>94</v>
       </c>
@@ -2123,7 +2281,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16">
       <c r="A22" s="27"/>
       <c r="B22" s="11">
         <f>1*$A$4</f>
@@ -2132,14 +2290,14 @@
       <c r="C22" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="44"/>
       <c r="J22" s="10" t="s">
         <v>99</v>
       </c>
@@ -2163,7 +2321,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="21">
       <c r="A23" s="27"/>
       <c r="B23" s="11">
         <f>1*$A$4</f>
@@ -2172,14 +2330,14 @@
       <c r="C23" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="41" t="s">
+      <c r="D23" s="42" t="s">
         <v>106</v>
       </c>
-      <c r="E23" s="42"/>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="43"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="43"/>
+      <c r="I23" s="44"/>
       <c r="J23" s="8" t="s">
         <v>105</v>
       </c>
@@ -2203,7 +2361,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" ht="21">
       <c r="A24" s="27"/>
       <c r="B24" s="11">
         <f>3*$A$4</f>
@@ -2212,14 +2370,14 @@
       <c r="C24" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="49" t="s">
+      <c r="D24" s="48" t="s">
         <v>110</v>
       </c>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="50"/>
-      <c r="I24" s="51"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="50"/>
       <c r="J24" s="8" t="s">
         <v>108</v>
       </c>
@@ -2243,7 +2401,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="21">
       <c r="A25" s="27"/>
       <c r="B25" s="11">
         <f>1*$A$4</f>
@@ -2252,14 +2410,14 @@
       <c r="C25" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="49" t="s">
+      <c r="D25" s="48" t="s">
         <v>115</v>
       </c>
-      <c r="E25" s="50"/>
-      <c r="F25" s="50"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="50"/>
-      <c r="I25" s="51"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="50"/>
       <c r="J25" s="8" t="s">
         <v>113</v>
       </c>
@@ -2283,7 +2441,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" ht="21">
       <c r="A26" s="27"/>
       <c r="B26" s="11">
         <f t="shared" ref="B26:B36" si="3">1*$A$4</f>
@@ -2292,14 +2450,14 @@
       <c r="C26" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D26" s="41" t="s">
+      <c r="D26" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="E26" s="42"/>
-      <c r="F26" s="42"/>
-      <c r="G26" s="42"/>
-      <c r="H26" s="42"/>
-      <c r="I26" s="43"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="43"/>
+      <c r="H26" s="43"/>
+      <c r="I26" s="44"/>
       <c r="J26" s="8" t="s">
         <v>117</v>
       </c>
@@ -2323,7 +2481,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16">
       <c r="A27" s="27"/>
       <c r="B27" s="11">
         <f>2*$A$4</f>
@@ -2332,14 +2490,14 @@
       <c r="C27" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="E27" s="42"/>
-      <c r="F27" s="42"/>
-      <c r="G27" s="42"/>
-      <c r="H27" s="42"/>
-      <c r="I27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="43"/>
+      <c r="I27" s="44"/>
       <c r="J27" s="10" t="s">
         <v>120</v>
       </c>
@@ -2363,7 +2521,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="21">
       <c r="A28" s="27"/>
       <c r="B28" s="11">
         <f t="shared" si="3"/>
@@ -2372,14 +2530,14 @@
       <c r="C28" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="E28" s="42"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42"/>
-      <c r="H28" s="42"/>
-      <c r="I28" s="43"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="43"/>
+      <c r="H28" s="43"/>
+      <c r="I28" s="44"/>
       <c r="J28" s="8" t="s">
         <v>126</v>
       </c>
@@ -2403,7 +2561,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16">
       <c r="A29" s="27"/>
       <c r="B29" s="11">
         <f t="shared" si="3"/>
@@ -2412,14 +2570,14 @@
       <c r="C29" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="42" t="s">
         <v>129</v>
       </c>
-      <c r="E29" s="42"/>
-      <c r="F29" s="42"/>
-      <c r="G29" s="42"/>
-      <c r="H29" s="42"/>
-      <c r="I29" s="43"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="43"/>
+      <c r="G29" s="43"/>
+      <c r="H29" s="43"/>
+      <c r="I29" s="44"/>
       <c r="J29" s="10" t="s">
         <v>130</v>
       </c>
@@ -2443,7 +2601,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="21">
       <c r="A30" s="27"/>
       <c r="B30" s="11">
         <f t="shared" si="3"/>
@@ -2452,14 +2610,14 @@
       <c r="C30" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="42" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="42"/>
-      <c r="F30" s="42"/>
-      <c r="G30" s="42"/>
-      <c r="H30" s="42"/>
-      <c r="I30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+      <c r="H30" s="43"/>
+      <c r="I30" s="44"/>
       <c r="J30" s="8" t="s">
         <v>134</v>
       </c>
@@ -2483,7 +2641,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="21">
       <c r="A31" s="27"/>
       <c r="B31" s="11">
         <f>7*$A$4</f>
@@ -2492,14 +2650,14 @@
       <c r="C31" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D31" s="49" t="s">
+      <c r="D31" s="48" t="s">
         <v>137</v>
       </c>
-      <c r="E31" s="50"/>
-      <c r="F31" s="50"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="51"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="49"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="49"/>
+      <c r="I31" s="50"/>
       <c r="J31" s="8" t="s">
         <v>138</v>
       </c>
@@ -2523,7 +2681,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="21">
       <c r="A32" s="27"/>
       <c r="B32" s="11">
         <f>2*$A$4</f>
@@ -2532,14 +2690,14 @@
       <c r="C32" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D32" s="41" t="s">
+      <c r="D32" s="42" t="s">
         <v>143</v>
       </c>
-      <c r="E32" s="42"/>
-      <c r="F32" s="42"/>
-      <c r="G32" s="42"/>
-      <c r="H32" s="42"/>
-      <c r="I32" s="43"/>
+      <c r="E32" s="43"/>
+      <c r="F32" s="43"/>
+      <c r="G32" s="43"/>
+      <c r="H32" s="43"/>
+      <c r="I32" s="44"/>
       <c r="J32" s="10">
         <v>1711725</v>
       </c>
@@ -2563,7 +2721,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" ht="21">
       <c r="A33" s="27"/>
       <c r="B33" s="11">
         <f t="shared" si="3"/>
@@ -2572,14 +2730,14 @@
       <c r="C33" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D33" s="41" t="s">
+      <c r="D33" s="42" t="s">
         <v>145</v>
       </c>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="43"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="43"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="43"/>
+      <c r="I33" s="44"/>
       <c r="J33" s="10" t="s">
         <v>147</v>
       </c>
@@ -2603,7 +2761,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16">
       <c r="A34" s="27"/>
       <c r="B34" s="11">
         <f t="shared" si="3"/>
@@ -2612,14 +2770,14 @@
       <c r="C34" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D34" s="41" t="s">
+      <c r="D34" s="42" t="s">
         <v>152</v>
       </c>
-      <c r="E34" s="42"/>
-      <c r="F34" s="42"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="42"/>
-      <c r="I34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="43"/>
+      <c r="H34" s="43"/>
+      <c r="I34" s="44"/>
       <c r="J34" s="10" t="s">
         <v>150</v>
       </c>
@@ -2643,7 +2801,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16">
       <c r="A35" s="27"/>
       <c r="B35" s="11">
         <f t="shared" si="3"/>
@@ -2652,14 +2810,14 @@
       <c r="C35" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D35" s="41" t="s">
+      <c r="D35" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="E35" s="42"/>
-      <c r="F35" s="42"/>
-      <c r="G35" s="42"/>
-      <c r="H35" s="42"/>
-      <c r="I35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="44"/>
       <c r="J35" s="10" t="s">
         <v>155</v>
       </c>
@@ -2683,7 +2841,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" ht="21" thickBot="1">
       <c r="A36" s="27"/>
       <c r="B36" s="35">
         <f t="shared" si="3"/>
@@ -2692,14 +2850,14 @@
       <c r="C36" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="D36" s="54" t="s">
+      <c r="D36" s="45" t="s">
         <v>159</v>
       </c>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
-      <c r="G36" s="55"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="56"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="46"/>
+      <c r="I36" s="47"/>
       <c r="J36" s="37" t="s">
         <v>158</v>
       </c>
@@ -2723,7 +2881,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16">
       <c r="A37" s="25">
         <v>4</v>
       </c>
@@ -2734,14 +2892,14 @@
       <c r="C37" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="44" t="s">
+      <c r="D37" s="55" t="s">
         <v>176</v>
       </c>
-      <c r="E37" s="45"/>
-      <c r="F37" s="45"/>
-      <c r="G37" s="45"/>
-      <c r="H37" s="45"/>
-      <c r="I37" s="46"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="57"/>
       <c r="J37" s="32" t="s">
         <v>165</v>
       </c>
@@ -2758,12 +2916,12 @@
         <v>3.1899999999999998E-2</v>
       </c>
       <c r="O37" s="22">
-        <f t="shared" ref="O37:O43" si="5">N37*B37</f>
+        <f t="shared" ref="O37:O46" si="5">N37*B37</f>
         <v>0.12759999999999999</v>
       </c>
       <c r="P37" s="34"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16">
       <c r="A38" s="25"/>
       <c r="B38" s="11">
         <f t="shared" ref="B38:B43" si="6">1*$A$37</f>
@@ -2772,14 +2930,14 @@
       <c r="C38" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="41" t="s">
+      <c r="D38" s="42" t="s">
         <v>178</v>
       </c>
-      <c r="E38" s="42"/>
-      <c r="F38" s="42"/>
-      <c r="G38" s="42"/>
-      <c r="H38" s="42"/>
-      <c r="I38" s="43"/>
+      <c r="E38" s="43"/>
+      <c r="F38" s="43"/>
+      <c r="G38" s="43"/>
+      <c r="H38" s="43"/>
+      <c r="I38" s="44"/>
       <c r="J38" s="28" t="s">
         <v>166</v>
       </c>
@@ -2801,7 +2959,7 @@
       </c>
       <c r="P38" s="15"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16">
       <c r="A39" s="25"/>
       <c r="B39" s="11">
         <f t="shared" si="6"/>
@@ -2810,14 +2968,14 @@
       <c r="C39" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D39" s="41" t="s">
+      <c r="D39" s="42" t="s">
         <v>182</v>
       </c>
-      <c r="E39" s="42"/>
-      <c r="F39" s="42"/>
-      <c r="G39" s="42"/>
-      <c r="H39" s="42"/>
-      <c r="I39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+      <c r="H39" s="43"/>
+      <c r="I39" s="44"/>
       <c r="J39" s="28" t="s">
         <v>167</v>
       </c>
@@ -2839,7 +2997,7 @@
       </c>
       <c r="P39" s="15"/>
     </row>
-    <row r="40" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" ht="21">
       <c r="A40" s="25"/>
       <c r="B40" s="11">
         <f t="shared" si="6"/>
@@ -2848,14 +3006,14 @@
       <c r="C40" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D40" s="41" t="s">
+      <c r="D40" s="42" t="s">
         <v>172</v>
       </c>
-      <c r="E40" s="42"/>
-      <c r="F40" s="42"/>
-      <c r="G40" s="42"/>
-      <c r="H40" s="42"/>
-      <c r="I40" s="43"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="43"/>
+      <c r="I40" s="44"/>
       <c r="J40" s="28" t="s">
         <v>168</v>
       </c>
@@ -2877,7 +3035,7 @@
       </c>
       <c r="P40" s="15"/>
     </row>
-    <row r="41" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" ht="21">
       <c r="A41" s="25"/>
       <c r="B41" s="11">
         <f>2*$A$37</f>
@@ -2886,14 +3044,14 @@
       <c r="C41" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D41" s="41" t="s">
+      <c r="D41" s="42" t="s">
         <v>173</v>
       </c>
-      <c r="E41" s="42"/>
-      <c r="F41" s="42"/>
-      <c r="G41" s="42"/>
-      <c r="H41" s="42"/>
-      <c r="I41" s="43"/>
+      <c r="E41" s="43"/>
+      <c r="F41" s="43"/>
+      <c r="G41" s="43"/>
+      <c r="H41" s="43"/>
+      <c r="I41" s="44"/>
       <c r="J41" s="28" t="s">
         <v>169</v>
       </c>
@@ -2915,7 +3073,7 @@
       </c>
       <c r="P41" s="15"/>
     </row>
-    <row r="42" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" ht="21">
       <c r="A42" s="25"/>
       <c r="B42" s="11">
         <f>2*$A$37</f>
@@ -2924,14 +3082,14 @@
       <c r="C42" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D42" s="41" t="s">
+      <c r="D42" s="42" t="s">
         <v>174</v>
       </c>
-      <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
-      <c r="H42" s="42"/>
-      <c r="I42" s="43"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="43"/>
+      <c r="G42" s="43"/>
+      <c r="H42" s="43"/>
+      <c r="I42" s="44"/>
       <c r="J42" s="28" t="s">
         <v>170</v>
       </c>
@@ -2953,7 +3111,7 @@
       </c>
       <c r="P42" s="15"/>
     </row>
-    <row r="43" spans="1:16" ht="17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" ht="21">
       <c r="A43" s="25"/>
       <c r="B43" s="11">
         <f t="shared" si="6"/>
@@ -2962,14 +3120,14 @@
       <c r="C43" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D43" s="41" t="s">
+      <c r="D43" s="42" t="s">
         <v>175</v>
       </c>
-      <c r="E43" s="42"/>
-      <c r="F43" s="42"/>
-      <c r="G43" s="42"/>
-      <c r="H43" s="42"/>
-      <c r="I43" s="43"/>
+      <c r="E43" s="43"/>
+      <c r="F43" s="43"/>
+      <c r="G43" s="43"/>
+      <c r="H43" s="43"/>
+      <c r="I43" s="44"/>
       <c r="J43" s="28" t="s">
         <v>171</v>
       </c>
@@ -2991,161 +3149,273 @@
       </c>
       <c r="P43" s="15"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="M44" s="23" t="s">
+    <row r="44" spans="1:16" ht="21">
+      <c r="A44" s="58">
         <v>5</v>
       </c>
-      <c r="N44" s="24"/>
-      <c r="O44" s="3">
-        <f>SUM(O4:O43)</f>
-        <v>110.7058</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B45" t="s">
+      <c r="B44" s="11">
+        <f>1*A44</f>
+        <v>5</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="D44" s="42" t="s">
+        <v>190</v>
+      </c>
+      <c r="E44" s="43"/>
+      <c r="F44" s="43"/>
+      <c r="G44" s="43"/>
+      <c r="H44" s="43"/>
+      <c r="I44" s="44"/>
+      <c r="J44" s="59" t="s">
+        <v>193</v>
+      </c>
+      <c r="K44" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="L44" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="M44" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="N44" s="29">
+        <v>1.73</v>
+      </c>
+      <c r="O44" s="13">
+        <f t="shared" si="5"/>
+        <v>8.65</v>
+      </c>
+      <c r="P44" s="15" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="21">
+      <c r="A45" s="58"/>
+      <c r="B45" s="11">
+        <f>1*A44</f>
+        <v>5</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="D45" s="42" t="s">
+        <v>191</v>
+      </c>
+      <c r="E45" s="43"/>
+      <c r="F45" s="43"/>
+      <c r="G45" s="43"/>
+      <c r="H45" s="43"/>
+      <c r="I45" s="44"/>
+      <c r="J45" s="60" t="s">
+        <v>194</v>
+      </c>
+      <c r="K45" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="L45" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="M45" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="N45" s="29">
+        <v>1.27</v>
+      </c>
+      <c r="O45" s="13">
+        <f t="shared" si="5"/>
+        <v>6.35</v>
+      </c>
+      <c r="P45" s="15" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="21">
+      <c r="A46" s="58"/>
+      <c r="B46" s="11">
+        <f>1*A44</f>
+        <v>5</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="D46" s="42" t="s">
+        <v>192</v>
+      </c>
+      <c r="E46" s="43"/>
+      <c r="F46" s="43"/>
+      <c r="G46" s="43"/>
+      <c r="H46" s="43"/>
+      <c r="I46" s="44"/>
+      <c r="J46" s="59" t="s">
+        <v>195</v>
+      </c>
+      <c r="K46" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="L46" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="M46" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="N46" s="29">
+        <v>0.27800000000000002</v>
+      </c>
+      <c r="O46" s="13">
+        <f t="shared" si="5"/>
+        <v>1.3900000000000001</v>
+      </c>
+      <c r="P46" s="15" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16">
+      <c r="M47" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="N47" s="24"/>
+      <c r="O47" s="3">
+        <f>SUM(O4:O46)</f>
+        <v>127.0958</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16">
+      <c r="B48" t="s">
         <v>7</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C48" t="s">
         <v>8</v>
       </c>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5"/>
-      <c r="L45" s="7"/>
-      <c r="M45" s="52" t="s">
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
+      <c r="L48" s="7"/>
+      <c r="M48" s="53" t="s">
         <v>162</v>
       </c>
-      <c r="N45" s="53"/>
-      <c r="O45" s="2"/>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B46" t="s">
+      <c r="N48" s="54"/>
+      <c r="O48" s="2"/>
+    </row>
+    <row r="49" spans="2:15">
+      <c r="B49" t="s">
         <v>10</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C49" t="s">
         <v>11</v>
       </c>
-      <c r="F46" s="4"/>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
-      <c r="I46" s="5"/>
-      <c r="J46" s="5"/>
-      <c r="K46" s="5"/>
-      <c r="L46" s="5"/>
-      <c r="M46" s="47" t="s">
+      <c r="F49" s="4"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+      <c r="L49" s="5"/>
+      <c r="M49" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="N46" s="47"/>
-      <c r="O46" s="6">
-        <f>O45+O44</f>
-        <v>110.7058</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="M47" s="16" t="s">
+      <c r="N49" s="51"/>
+      <c r="O49" s="6">
+        <f>O48+O47</f>
+        <v>127.0958</v>
+      </c>
+    </row>
+    <row r="50" spans="2:15">
+      <c r="M50" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="O47" s="17">
-        <f>O46/5</f>
-        <v>22.141159999999999</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="M48" t="s">
+      <c r="O50" s="17">
+        <f>O49/5</f>
+        <v>25.419159999999998</v>
+      </c>
+    </row>
+    <row r="51" spans="2:15">
+      <c r="M51" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="49" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="M49" s="16" t="s">
+    <row r="52" spans="2:15">
+      <c r="M52" s="16" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="50" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="M50" t="s">
+    <row r="53" spans="2:15">
+      <c r="M53" t="s">
         <v>39</v>
       </c>
-      <c r="N50" s="57">
+      <c r="N53" s="41">
         <v>116.94</v>
       </c>
     </row>
-    <row r="51" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="M51" t="s">
+    <row r="54" spans="2:15">
+      <c r="M54" t="s">
         <v>100</v>
       </c>
-      <c r="N51" s="57">
+      <c r="N54" s="41">
         <v>22.43</v>
       </c>
     </row>
-    <row r="52" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="M52" t="s">
+    <row r="55" spans="2:15">
+      <c r="M55" t="s">
         <v>163</v>
       </c>
-      <c r="N52" s="57">
+      <c r="N55" s="41">
         <v>18.690000000000001</v>
       </c>
     </row>
-    <row r="53" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="N53" s="57">
-        <f>SUM(N50:N52)</f>
+    <row r="56" spans="2:15">
+      <c r="N56" s="41">
+        <f>SUM(N53:N55)</f>
         <v>158.06</v>
       </c>
     </row>
-    <row r="55" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="M55" s="16" t="s">
+    <row r="58" spans="2:15">
+      <c r="M58" s="16" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="56" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="M56" t="s">
-        <v>16</v>
-      </c>
-      <c r="N56" s="57">
+    <row r="59" spans="2:15">
+      <c r="M59" t="s">
+        <v>16</v>
+      </c>
+      <c r="N59" s="41">
         <v>5.24</v>
       </c>
     </row>
-    <row r="57" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="M57" t="s">
+    <row r="60" spans="2:15">
+      <c r="M60" t="s">
         <v>163</v>
       </c>
-      <c r="N57" s="57">
+      <c r="N60" s="41">
         <v>15.76</v>
       </c>
     </row>
-    <row r="58" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="N58" s="57">
-        <f>SUM(N56:N57)</f>
+    <row r="61" spans="2:15">
+      <c r="N61" s="41">
+        <f>SUM(N59:N60)</f>
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="13:14" x14ac:dyDescent="0.2">
-      <c r="N59" s="21"/>
+    <row r="62" spans="2:15">
+      <c r="N62" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="43">
-    <mergeCell ref="D32:I32"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="D34:I34"/>
-    <mergeCell ref="D35:I35"/>
-    <mergeCell ref="D36:I36"/>
-    <mergeCell ref="D14:I14"/>
-    <mergeCell ref="D17:I17"/>
-    <mergeCell ref="D18:I18"/>
-    <mergeCell ref="D19:I19"/>
-    <mergeCell ref="D20:I20"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="D28:I28"/>
-    <mergeCell ref="D29:I29"/>
-    <mergeCell ref="D30:I30"/>
-    <mergeCell ref="D31:I31"/>
-    <mergeCell ref="D22:I22"/>
-    <mergeCell ref="D23:I23"/>
-    <mergeCell ref="D24:I24"/>
-    <mergeCell ref="D25:I25"/>
-    <mergeCell ref="D26:I26"/>
-    <mergeCell ref="M46:N46"/>
+  <mergeCells count="46">
+    <mergeCell ref="D44:I44"/>
+    <mergeCell ref="D45:I45"/>
+    <mergeCell ref="D46:I46"/>
+    <mergeCell ref="D42:I42"/>
+    <mergeCell ref="D43:I43"/>
+    <mergeCell ref="D37:I37"/>
+    <mergeCell ref="D38:I38"/>
+    <mergeCell ref="D39:I39"/>
+    <mergeCell ref="D40:I40"/>
+    <mergeCell ref="D41:I41"/>
+    <mergeCell ref="M49:N49"/>
     <mergeCell ref="D13:I13"/>
     <mergeCell ref="D3:I3"/>
     <mergeCell ref="D4:I4"/>
@@ -3157,18 +3427,32 @@
     <mergeCell ref="D10:I10"/>
     <mergeCell ref="D11:I11"/>
     <mergeCell ref="D12:I12"/>
-    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="M48:N48"/>
     <mergeCell ref="D16:I16"/>
     <mergeCell ref="D15:I15"/>
     <mergeCell ref="D21:I21"/>
-    <mergeCell ref="D42:I42"/>
-    <mergeCell ref="D43:I43"/>
-    <mergeCell ref="D37:I37"/>
-    <mergeCell ref="D38:I38"/>
-    <mergeCell ref="D39:I39"/>
-    <mergeCell ref="D40:I40"/>
-    <mergeCell ref="D41:I41"/>
+    <mergeCell ref="D22:I22"/>
+    <mergeCell ref="D23:I23"/>
+    <mergeCell ref="D24:I24"/>
+    <mergeCell ref="D25:I25"/>
+    <mergeCell ref="D26:I26"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="D28:I28"/>
+    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="D30:I30"/>
+    <mergeCell ref="D31:I31"/>
+    <mergeCell ref="D14:I14"/>
+    <mergeCell ref="D17:I17"/>
+    <mergeCell ref="D18:I18"/>
+    <mergeCell ref="D19:I19"/>
+    <mergeCell ref="D20:I20"/>
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="D34:I34"/>
+    <mergeCell ref="D35:I35"/>
+    <mergeCell ref="D36:I36"/>
   </mergeCells>
+  <phoneticPr fontId="6"/>
   <hyperlinks>
     <hyperlink ref="P5" r:id="rId1" xr:uid="{5644B2BA-ED03-8440-9B66-CBBFBD5F9484}"/>
     <hyperlink ref="P6" r:id="rId2" xr:uid="{59111D94-A944-E540-AFD1-58CECAA9E13F}"/>
@@ -3200,6 +3484,8 @@
     <hyperlink ref="P34" r:id="rId28" xr:uid="{23428F13-92D9-4C4B-BA09-C7E898976C23}"/>
     <hyperlink ref="P35" r:id="rId29" xr:uid="{B1937385-999A-4F41-9FC8-1C5A0D27E01A}"/>
     <hyperlink ref="P36" r:id="rId30" xr:uid="{EABDE385-3109-9243-A76B-B995D48E36D4}"/>
+    <hyperlink ref="P44" r:id="rId31" xr:uid="{FC5066C6-93D7-DE42-82DA-765A7F3023A6}"/>
+    <hyperlink ref="P46" r:id="rId32" xr:uid="{A6173A0A-F7EF-4E42-BDAE-A6954C6DC48E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>